<commit_message>
Rename 'API' column to 'Sales Data'
</commit_message>
<xml_diff>
--- a/Brand_Document_Tracker (1).xlsx
+++ b/Brand_Document_Tracker (1).xlsx
@@ -124,7 +124,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -191,11 +191,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -283,6 +327,8 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -697,7 +743,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>Sales Data</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
@@ -1187,7 +1233,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>API, Menu , Employee list , medical , police verification are left</t>
+          <t>Sales Data, Menu, Employee list, medical, police verification are left</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1471,22 +1517,13 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="22" t="inlineStr">
         <is>
           <t>BRAND-WISE PENDING ITEMS</t>
         </is>
       </c>
-      <c r="C16" s="23" t="n"/>
-      <c r="D16" s="23" t="n"/>
-      <c r="E16" s="23" t="n"/>
-      <c r="F16" s="23" t="n"/>
-      <c r="G16" s="23" t="n"/>
-      <c r="H16" s="23" t="n"/>
-      <c r="I16" s="23" t="n"/>
-      <c r="J16" s="23" t="n"/>
-      <c r="K16" s="23" t="n"/>
-      <c r="L16" s="23" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="24" t="inlineStr">
@@ -1499,14 +1536,6 @@
           <t>Pending Documents</t>
         </is>
       </c>
-      <c r="D17" s="25" t="n"/>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="25" t="n"/>
-      <c r="G17" s="25" t="n"/>
-      <c r="H17" s="25" t="n"/>
-      <c r="I17" s="25" t="n"/>
-      <c r="J17" s="25" t="n"/>
-      <c r="K17" s="25" t="n"/>
       <c r="L17" s="26" t="inlineStr">
         <is>
           <t>Count</t>
@@ -1524,14 +1553,14 @@
           <t>FSSAI (Applied), PDC</t>
         </is>
       </c>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="29" t="n"/>
-      <c r="F18" s="29" t="n"/>
-      <c r="G18" s="29" t="n"/>
-      <c r="H18" s="29" t="n"/>
-      <c r="I18" s="29" t="n"/>
-      <c r="J18" s="29" t="n"/>
-      <c r="K18" s="29" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="33" t="n"/>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="n"/>
+      <c r="I18" s="33" t="n"/>
+      <c r="J18" s="33" t="n"/>
+      <c r="K18" s="34" t="n"/>
       <c r="L18" s="30" t="n">
         <v>2</v>
       </c>
@@ -1547,14 +1576,14 @@
           <t>FSSAI (Applied), PDC, Police Verification</t>
         </is>
       </c>
-      <c r="D19" s="29" t="n"/>
-      <c r="E19" s="29" t="n"/>
-      <c r="F19" s="29" t="n"/>
-      <c r="G19" s="29" t="n"/>
-      <c r="H19" s="29" t="n"/>
-      <c r="I19" s="29" t="n"/>
-      <c r="J19" s="29" t="n"/>
-      <c r="K19" s="29" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
+      <c r="G19" s="33" t="n"/>
+      <c r="H19" s="33" t="n"/>
+      <c r="I19" s="33" t="n"/>
+      <c r="J19" s="33" t="n"/>
+      <c r="K19" s="34" t="n"/>
       <c r="L19" s="30" t="n">
         <v>3</v>
       </c>
@@ -1567,17 +1596,17 @@
       </c>
       <c r="C20" s="28" t="inlineStr">
         <is>
-          <t>Term Sheet, Agreement, FSSAI, API, Menu, PDC, Employee List, Medical, Police Verification</t>
-        </is>
-      </c>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="29" t="n"/>
-      <c r="F20" s="29" t="n"/>
-      <c r="G20" s="29" t="n"/>
-      <c r="H20" s="29" t="n"/>
-      <c r="I20" s="29" t="n"/>
-      <c r="J20" s="29" t="n"/>
-      <c r="K20" s="29" t="n"/>
+          <t>Term Sheet, Agreement, FSSAI, Sales Data, Menu, PDC, Employee List, Medical, Police Verification</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="n"/>
+      <c r="I20" s="33" t="n"/>
+      <c r="J20" s="33" t="n"/>
+      <c r="K20" s="34" t="n"/>
       <c r="L20" s="30" t="n">
         <v>9</v>
       </c>
@@ -1590,17 +1619,17 @@
       </c>
       <c r="C21" s="28" t="inlineStr">
         <is>
-          <t>API, PDC</t>
-        </is>
-      </c>
-      <c r="D21" s="29" t="n"/>
-      <c r="E21" s="29" t="n"/>
-      <c r="F21" s="29" t="n"/>
-      <c r="G21" s="29" t="n"/>
-      <c r="H21" s="29" t="n"/>
-      <c r="I21" s="29" t="n"/>
-      <c r="J21" s="29" t="n"/>
-      <c r="K21" s="29" t="n"/>
+          <t>Sales Data, PDC</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="n"/>
+      <c r="I21" s="33" t="n"/>
+      <c r="J21" s="33" t="n"/>
+      <c r="K21" s="34" t="n"/>
       <c r="L21" s="30" t="n">
         <v>2</v>
       </c>
@@ -1613,17 +1642,17 @@
       </c>
       <c r="C22" s="28" t="inlineStr">
         <is>
-          <t>Agreement, FSSAI, API, PDC, Medical, Police Verification</t>
-        </is>
-      </c>
-      <c r="D22" s="29" t="n"/>
-      <c r="E22" s="29" t="n"/>
-      <c r="F22" s="29" t="n"/>
-      <c r="G22" s="29" t="n"/>
-      <c r="H22" s="29" t="n"/>
-      <c r="I22" s="29" t="n"/>
-      <c r="J22" s="29" t="n"/>
-      <c r="K22" s="29" t="n"/>
+          <t>Agreement, FSSAI, Sales Data, PDC, Medical, Police Verification</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="n"/>
+      <c r="I22" s="33" t="n"/>
+      <c r="J22" s="33" t="n"/>
+      <c r="K22" s="34" t="n"/>
       <c r="L22" s="30" t="n">
         <v>6</v>
       </c>
@@ -1636,17 +1665,17 @@
       </c>
       <c r="C23" s="28" t="inlineStr">
         <is>
-          <t>Term Sheet, Agreement, FSSAI, API, Menu, PDC, Employee List, Medical, Police Verification</t>
-        </is>
-      </c>
-      <c r="D23" s="29" t="n"/>
-      <c r="E23" s="29" t="n"/>
-      <c r="F23" s="29" t="n"/>
-      <c r="G23" s="29" t="n"/>
-      <c r="H23" s="29" t="n"/>
-      <c r="I23" s="29" t="n"/>
-      <c r="J23" s="29" t="n"/>
-      <c r="K23" s="29" t="n"/>
+          <t>Term Sheet, Agreement, FSSAI, Sales Data, Menu, PDC, Employee List, Medical, Police Verification</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="n"/>
+      <c r="I23" s="33" t="n"/>
+      <c r="J23" s="33" t="n"/>
+      <c r="K23" s="34" t="n"/>
       <c r="L23" s="30" t="n">
         <v>9</v>
       </c>
@@ -1659,17 +1688,17 @@
       </c>
       <c r="C24" s="28" t="inlineStr">
         <is>
-          <t>API, Employee List, Medical, Police Verification, Mail not sent</t>
-        </is>
-      </c>
-      <c r="D24" s="29" t="n"/>
-      <c r="E24" s="29" t="n"/>
-      <c r="F24" s="29" t="n"/>
-      <c r="G24" s="29" t="n"/>
-      <c r="H24" s="29" t="n"/>
-      <c r="I24" s="29" t="n"/>
-      <c r="J24" s="29" t="n"/>
-      <c r="K24" s="29" t="n"/>
+          <t>Sales Data, Employee List, Medical, Police Verification, Mail not sent</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="33" t="n"/>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="33" t="n"/>
+      <c r="I24" s="33" t="n"/>
+      <c r="J24" s="33" t="n"/>
+      <c r="K24" s="34" t="n"/>
       <c r="L24" s="30" t="n">
         <v>5</v>
       </c>
@@ -1685,14 +1714,14 @@
           <t>PDC, Police Verification</t>
         </is>
       </c>
-      <c r="D25" s="29" t="n"/>
-      <c r="E25" s="29" t="n"/>
-      <c r="F25" s="29" t="n"/>
-      <c r="G25" s="29" t="n"/>
-      <c r="H25" s="29" t="n"/>
-      <c r="I25" s="29" t="n"/>
-      <c r="J25" s="29" t="n"/>
-      <c r="K25" s="29" t="n"/>
+      <c r="D25" s="33" t="n"/>
+      <c r="E25" s="33" t="n"/>
+      <c r="F25" s="33" t="n"/>
+      <c r="G25" s="33" t="n"/>
+      <c r="H25" s="33" t="n"/>
+      <c r="I25" s="33" t="n"/>
+      <c r="J25" s="33" t="n"/>
+      <c r="K25" s="34" t="n"/>
       <c r="L25" s="30" t="n">
         <v>2</v>
       </c>
@@ -1705,17 +1734,17 @@
       </c>
       <c r="C26" s="28" t="inlineStr">
         <is>
-          <t>Term Sheet, Agreement, FSSAI, API, Menu, PDC, Employee List, Medical, Police Verification</t>
-        </is>
-      </c>
-      <c r="D26" s="29" t="n"/>
-      <c r="E26" s="29" t="n"/>
-      <c r="F26" s="29" t="n"/>
-      <c r="G26" s="29" t="n"/>
-      <c r="H26" s="29" t="n"/>
-      <c r="I26" s="29" t="n"/>
-      <c r="J26" s="29" t="n"/>
-      <c r="K26" s="29" t="n"/>
+          <t>Term Sheet, Agreement, FSSAI, Sales Data, Menu, PDC, Employee List, Medical, Police Verification</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="n"/>
+      <c r="E26" s="33" t="n"/>
+      <c r="F26" s="33" t="n"/>
+      <c r="G26" s="33" t="n"/>
+      <c r="H26" s="33" t="n"/>
+      <c r="I26" s="33" t="n"/>
+      <c r="J26" s="33" t="n"/>
+      <c r="K26" s="34" t="n"/>
       <c r="L26" s="30" t="n">
         <v>9</v>
       </c>
@@ -1731,14 +1760,14 @@
           <t>Term Sheet, Menu, PDC, Employee List, Medical, Police Verification</t>
         </is>
       </c>
-      <c r="D27" s="29" t="n"/>
-      <c r="E27" s="29" t="n"/>
-      <c r="F27" s="29" t="n"/>
-      <c r="G27" s="29" t="n"/>
-      <c r="H27" s="29" t="n"/>
-      <c r="I27" s="29" t="n"/>
-      <c r="J27" s="29" t="n"/>
-      <c r="K27" s="29" t="n"/>
+      <c r="D27" s="33" t="n"/>
+      <c r="E27" s="33" t="n"/>
+      <c r="F27" s="33" t="n"/>
+      <c r="G27" s="33" t="n"/>
+      <c r="H27" s="33" t="n"/>
+      <c r="I27" s="33" t="n"/>
+      <c r="J27" s="33" t="n"/>
+      <c r="K27" s="34" t="n"/>
       <c r="L27" s="30" t="n">
         <v>6</v>
       </c>
@@ -1754,18 +1783,19 @@
           <t>Term Sheet, Agreement, FSSAI, Menu, PDC, Employee List, Medical, Police Verification</t>
         </is>
       </c>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="29" t="n"/>
-      <c r="F28" s="29" t="n"/>
-      <c r="G28" s="29" t="n"/>
-      <c r="H28" s="29" t="n"/>
-      <c r="I28" s="29" t="n"/>
-      <c r="J28" s="29" t="n"/>
-      <c r="K28" s="29" t="n"/>
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="33" t="n"/>
+      <c r="F28" s="33" t="n"/>
+      <c r="G28" s="33" t="n"/>
+      <c r="H28" s="33" t="n"/>
+      <c r="I28" s="33" t="n"/>
+      <c r="J28" s="33" t="n"/>
+      <c r="K28" s="34" t="n"/>
       <c r="L28" s="30" t="n">
         <v>8</v>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="B30" s="31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Treat 'A' status as Done (green); remove Applied from summary and legend
</commit_message>
<xml_diff>
--- a/Brand_Document_Tracker (1).xlsx
+++ b/Brand_Document_Tracker (1).xlsx
@@ -239,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -329,6 +329,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -796,9 +799,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -866,9 +869,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -1550,7 +1553,7 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>FSSAI (Applied), PDC</t>
+          <t>PDC</t>
         </is>
       </c>
       <c r="D18" s="33" t="n"/>
@@ -1562,7 +1565,7 @@
       <c r="J18" s="33" t="n"/>
       <c r="K18" s="34" t="n"/>
       <c r="L18" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" s="13">
@@ -1573,7 +1576,7 @@
       </c>
       <c r="C19" s="28" t="inlineStr">
         <is>
-          <t>FSSAI (Applied), PDC, Police Verification</t>
+          <t>PDC, Police Verification</t>
         </is>
       </c>
       <c r="D19" s="33" t="n"/>
@@ -1585,7 +1588,7 @@
       <c r="J19" s="33" t="n"/>
       <c r="K19" s="34" t="n"/>
       <c r="L19" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" s="13">
@@ -1812,11 +1815,7 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="E30" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
+      <c r="E30" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">

</xml_diff>